<commit_message>
SetJudge and Id openXML
</commit_message>
<xml_diff>
--- a/mallar/Protokoll/Protokoll_2019_lag_sv-r_mellan(mall).xlsx
+++ b/mallar/Protokoll/Protokoll_2019_lag_sv-r_mellan(mall).xlsx
@@ -1,123 +1,123 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28526"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<x:workbook xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <x:fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28526"/>
+  <x:workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\episerver\voltige\VoltigeClosedXML\mallar\Protokoll\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D54E0CEE-B78A-46E4-8FB4-DD51AEAB4E7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="43080" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Information" sheetId="27" r:id="rId1"/>
-    <sheet name="Häst, lag" sheetId="30" r:id="rId2"/>
-    <sheet name="Lag grund A" sheetId="22" r:id="rId3"/>
-    <sheet name="Lag grund D" sheetId="17" r:id="rId4"/>
-    <sheet name="Lag grund B" sheetId="18" r:id="rId5"/>
-    <sheet name="Lag kür tekn mellan" sheetId="29" r:id="rId6"/>
-    <sheet name="Lag kür tekn junior" sheetId="6" r:id="rId7"/>
-    <sheet name="Lag kür tekn sr" sheetId="20" r:id="rId8"/>
-    <sheet name="Lag kür art" sheetId="21" r:id="rId9"/>
-    <sheet name="Lag kür art senior" sheetId="31" r:id="rId10"/>
-  </sheets>
-  <externalReferences>
-    <externalReference r:id="rId11"/>
-    <externalReference r:id="rId12"/>
-  </externalReferences>
-  <definedNames>
-    <definedName name="Antal_tävlingsdagar" localSheetId="1">[1]Information!$H$5</definedName>
-    <definedName name="Antal_tävlingsdagar">[2]Information!$H$5</definedName>
-    <definedName name="bord" localSheetId="1">'Häst, lag'!$K$3</definedName>
-    <definedName name="bord" localSheetId="2">'Lag grund A'!$L$3</definedName>
-    <definedName name="bord" localSheetId="4">'Lag grund B'!$L$3</definedName>
-    <definedName name="bord" localSheetId="3">'Lag grund D'!$L$3</definedName>
-    <definedName name="bord" localSheetId="8">'Lag kür art'!$L$3</definedName>
-    <definedName name="bord" localSheetId="9">'Lag kür art senior'!$L$3</definedName>
-    <definedName name="bord" localSheetId="6">'Lag kür tekn junior'!$L$3</definedName>
-    <definedName name="bord" localSheetId="5">'Lag kür tekn mellan'!$L$3</definedName>
-    <definedName name="bord" localSheetId="7">'Lag kür tekn sr'!$L$3</definedName>
-    <definedName name="datum" localSheetId="1">'Häst, lag'!$C$4</definedName>
-    <definedName name="datum" localSheetId="2">'Lag grund A'!$C$4</definedName>
-    <definedName name="datum" localSheetId="4">'Lag grund B'!$C$4</definedName>
-    <definedName name="datum" localSheetId="3">'Lag grund D'!$C$4</definedName>
-    <definedName name="datum" localSheetId="8">'Lag kür art'!$C$4</definedName>
-    <definedName name="datum" localSheetId="9">'Lag kür art senior'!$C$4</definedName>
-    <definedName name="datum" localSheetId="6">'Lag kür tekn junior'!$C$4</definedName>
-    <definedName name="datum" localSheetId="5">'Lag kür tekn mellan'!$C$4</definedName>
-    <definedName name="datum" localSheetId="7">'Lag kür tekn sr'!$C$4</definedName>
-    <definedName name="domare" localSheetId="1">'Häst, lag'!$C$36</definedName>
-    <definedName name="domare" localSheetId="2">'Lag grund A'!$C$33</definedName>
-    <definedName name="domare" localSheetId="4">'Lag grund B'!$C$32</definedName>
-    <definedName name="domare" localSheetId="3">'Lag grund D'!$C$33</definedName>
-    <definedName name="domare" localSheetId="8">'Lag kür art'!$C$27</definedName>
-    <definedName name="domare" localSheetId="9">'Lag kür art senior'!$C$27</definedName>
-    <definedName name="domare" localSheetId="6">'Lag kür tekn junior'!$C$42</definedName>
-    <definedName name="domare" localSheetId="5">'Lag kür tekn mellan'!$C$42</definedName>
-    <definedName name="domare" localSheetId="7">'Lag kür tekn sr'!$C$42</definedName>
-    <definedName name="firstvaulter" localSheetId="1">'Häst, lag'!$H$7</definedName>
-    <definedName name="firstvaulter" localSheetId="2">'Lag grund A'!$I$7</definedName>
-    <definedName name="firstvaulter" localSheetId="4">'Lag grund B'!$I$7</definedName>
-    <definedName name="firstvaulter" localSheetId="3">'Lag grund D'!$I$7</definedName>
-    <definedName name="firstvaulter" localSheetId="8">'Lag kür art'!$I$7</definedName>
-    <definedName name="firstvaulter" localSheetId="9">'Lag kür art senior'!$I$7</definedName>
-    <definedName name="firstvaulter" localSheetId="6">'Lag kür tekn junior'!$I$7</definedName>
-    <definedName name="firstvaulter" localSheetId="5">'Lag kür tekn mellan'!$I$7</definedName>
-    <definedName name="firstvaulter" localSheetId="7">'Lag kür tekn sr'!$I$7</definedName>
-    <definedName name="header" localSheetId="1">'Häst, lag'!$A$2</definedName>
-    <definedName name="id" localSheetId="1">'Häst, lag'!$U$1</definedName>
-    <definedName name="id" localSheetId="2">'Lag grund A'!$U$1</definedName>
-    <definedName name="id" localSheetId="4">'Lag grund B'!$U$1</definedName>
-    <definedName name="id" localSheetId="3">'Lag grund D'!$U$1</definedName>
-    <definedName name="id" localSheetId="8">'Lag kür art'!$U$1</definedName>
-    <definedName name="id" localSheetId="9">'Lag kür art senior'!$U$1</definedName>
-    <definedName name="id" localSheetId="6">'Lag kür tekn junior'!$U$1</definedName>
-    <definedName name="id" localSheetId="5">'Lag kür tekn mellan'!$U$1</definedName>
-    <definedName name="id" localSheetId="7">'Lag kür tekn sr'!$U$1</definedName>
-    <definedName name="klass" localSheetId="1">'Häst, lag'!$K$4</definedName>
-    <definedName name="klass" localSheetId="2">'Lag grund A'!$L$4</definedName>
-    <definedName name="klass" localSheetId="4">'Lag grund B'!$L$4</definedName>
-    <definedName name="klass" localSheetId="3">'Lag grund D'!$L$4</definedName>
-    <definedName name="klass" localSheetId="8">'Lag kür art'!$L$4</definedName>
-    <definedName name="klass" localSheetId="9">'Lag kür art senior'!$L$4</definedName>
-    <definedName name="klass" localSheetId="6">'Lag kür tekn junior'!$L$4</definedName>
-    <definedName name="klass" localSheetId="5">'Lag kür tekn mellan'!$L$4</definedName>
-    <definedName name="klass" localSheetId="7">'Lag kür tekn sr'!$L$4</definedName>
-    <definedName name="moment" localSheetId="1">'Häst, lag'!$K$5</definedName>
-    <definedName name="moment" localSheetId="2">'Lag grund A'!$L$5</definedName>
-    <definedName name="moment" localSheetId="4">'Lag grund B'!$L$5</definedName>
-    <definedName name="moment" localSheetId="3">'Lag grund D'!$L$5</definedName>
-    <definedName name="moment" localSheetId="8">'Lag kür art'!$L$5</definedName>
-    <definedName name="moment" localSheetId="9">'Lag kür art senior'!$L$5</definedName>
-    <definedName name="moment" localSheetId="6">'Lag kür tekn junior'!$L$5</definedName>
-    <definedName name="moment" localSheetId="5">'Lag kür tekn mellan'!$L$5</definedName>
-    <definedName name="moment" localSheetId="7">'Lag kür tekn sr'!$L$5</definedName>
-    <definedName name="result" localSheetId="1">'Häst, lag'!$K$32</definedName>
-    <definedName name="result" localSheetId="2">'Lag grund A'!$L$29</definedName>
-    <definedName name="result" localSheetId="4">'Lag grund B'!$L$29</definedName>
-    <definedName name="result" localSheetId="3">'Lag grund D'!$L$29</definedName>
-    <definedName name="result" localSheetId="8">'Lag kür art'!$L$24</definedName>
-    <definedName name="result" localSheetId="9">'Lag kür art senior'!$L$24</definedName>
-    <definedName name="result" localSheetId="6">'Lag kür tekn junior'!$L$34</definedName>
-    <definedName name="result" localSheetId="5">'Lag kür tekn mellan'!$L$34</definedName>
-    <definedName name="result" localSheetId="7">'Lag kür tekn sr'!$L$35</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Häst, lag'!$A$1:$L$36</definedName>
-  </definedNames>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+  <x:bookViews>
+    <x:workbookView xWindow="43080" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </x:bookViews>
+  <x:sheets>
+    <x:sheet name="Information" sheetId="27" r:id="rId1"/>
+    <x:sheet name="Häst, lag" sheetId="30" r:id="rId2"/>
+    <x:sheet name="Lag grund A" sheetId="22" r:id="rId3"/>
+    <x:sheet name="Lag grund D" sheetId="17" r:id="rId4"/>
+    <x:sheet name="Lag grund B" sheetId="18" r:id="rId5"/>
+    <x:sheet name="Lag kür tekn mellan" sheetId="29" r:id="rId6"/>
+    <x:sheet name="Lag kür tekn junior" sheetId="6" r:id="rId7"/>
+    <x:sheet name="Lag kür tekn sr" sheetId="20" r:id="rId8"/>
+    <x:sheet name="Lag kür art" sheetId="21" r:id="rId9"/>
+    <x:sheet name="Lag kür art senior" sheetId="31" r:id="rId10"/>
+  </x:sheets>
+  <x:externalReferences>
+    <x:externalReference r:id="rId11"/>
+    <x:externalReference r:id="rId12"/>
+  </x:externalReferences>
+  <x:definedNames>
+    <x:definedName name="Antal_tävlingsdagar" localSheetId="1">[1]Information!$H$5</x:definedName>
+    <x:definedName name="Antal_tävlingsdagar">[2]Information!$H$5</x:definedName>
+    <x:definedName name="bord" localSheetId="1">'Häst, lag'!$K$3</x:definedName>
+    <x:definedName name="bord" localSheetId="2">'Lag grund A'!$L$3</x:definedName>
+    <x:definedName name="bord" localSheetId="4">'Lag grund B'!$L$3</x:definedName>
+    <x:definedName name="bord" localSheetId="3">'Lag grund D'!$L$3</x:definedName>
+    <x:definedName name="bord" localSheetId="8">'Lag kür art'!$L$3</x:definedName>
+    <x:definedName name="bord" localSheetId="9">'Lag kür art senior'!$L$3</x:definedName>
+    <x:definedName name="bord" localSheetId="6">'Lag kür tekn junior'!$L$3</x:definedName>
+    <x:definedName name="bord" localSheetId="5">'Lag kür tekn mellan'!$L$3</x:definedName>
+    <x:definedName name="bord" localSheetId="7">'Lag kür tekn sr'!$L$3</x:definedName>
+    <x:definedName name="datum" localSheetId="1">'Häst, lag'!$C$4</x:definedName>
+    <x:definedName name="datum" localSheetId="2">'Lag grund A'!$C$4</x:definedName>
+    <x:definedName name="datum" localSheetId="4">'Lag grund B'!$C$4</x:definedName>
+    <x:definedName name="datum" localSheetId="3">'Lag grund D'!$C$4</x:definedName>
+    <x:definedName name="datum" localSheetId="8">'Lag kür art'!$C$4</x:definedName>
+    <x:definedName name="datum" localSheetId="9">'Lag kür art senior'!$C$4</x:definedName>
+    <x:definedName name="datum" localSheetId="6">'Lag kür tekn junior'!$C$4</x:definedName>
+    <x:definedName name="datum" localSheetId="5">'Lag kür tekn mellan'!$C$4</x:definedName>
+    <x:definedName name="datum" localSheetId="7">'Lag kür tekn sr'!$C$4</x:definedName>
+    <x:definedName name="domare" localSheetId="1">'Häst, lag'!$C$36</x:definedName>
+    <x:definedName name="domare" localSheetId="2">'Lag grund A'!$C$33</x:definedName>
+    <x:definedName name="domare" localSheetId="4">'Lag grund B'!$C$32</x:definedName>
+    <x:definedName name="domare" localSheetId="3">'Lag grund D'!$C$33</x:definedName>
+    <x:definedName name="domare" localSheetId="8">'Lag kür art'!$C$27</x:definedName>
+    <x:definedName name="domare" localSheetId="9">'Lag kür art senior'!$C$27</x:definedName>
+    <x:definedName name="domare" localSheetId="6">'Lag kür tekn junior'!$C$42</x:definedName>
+    <x:definedName name="domare" localSheetId="5">'Lag kür tekn mellan'!$C$42</x:definedName>
+    <x:definedName name="domare" localSheetId="7">'Lag kür tekn sr'!$C$42</x:definedName>
+    <x:definedName name="firstvaulter" localSheetId="1">'Häst, lag'!$H$7</x:definedName>
+    <x:definedName name="firstvaulter" localSheetId="2">'Lag grund A'!$I$7</x:definedName>
+    <x:definedName name="firstvaulter" localSheetId="4">'Lag grund B'!$I$7</x:definedName>
+    <x:definedName name="firstvaulter" localSheetId="3">'Lag grund D'!$I$7</x:definedName>
+    <x:definedName name="firstvaulter" localSheetId="8">'Lag kür art'!$I$7</x:definedName>
+    <x:definedName name="firstvaulter" localSheetId="9">'Lag kür art senior'!$I$7</x:definedName>
+    <x:definedName name="firstvaulter" localSheetId="6">'Lag kür tekn junior'!$I$7</x:definedName>
+    <x:definedName name="firstvaulter" localSheetId="5">'Lag kür tekn mellan'!$I$7</x:definedName>
+    <x:definedName name="firstvaulter" localSheetId="7">'Lag kür tekn sr'!$I$7</x:definedName>
+    <x:definedName name="header" localSheetId="1">'Häst, lag'!$A$2</x:definedName>
+    <x:definedName name="id" localSheetId="1">'Häst, lag'!$U$1</x:definedName>
+    <x:definedName name="id" localSheetId="2">'Lag grund A'!$U$1</x:definedName>
+    <x:definedName name="id" localSheetId="4">'Lag grund B'!$U$1</x:definedName>
+    <x:definedName name="id" localSheetId="3">'Lag grund D'!$U$1</x:definedName>
+    <x:definedName name="id" localSheetId="8">'Lag kür art'!$U$1</x:definedName>
+    <x:definedName name="id" localSheetId="9">'Lag kür art senior'!$U$1</x:definedName>
+    <x:definedName name="id" localSheetId="6">'Lag kür tekn junior'!$U$1</x:definedName>
+    <x:definedName name="id" localSheetId="5">'Lag kür tekn mellan'!$U$1</x:definedName>
+    <x:definedName name="id" localSheetId="7">'Lag kür tekn sr'!$U$1</x:definedName>
+    <x:definedName name="klass" localSheetId="1">'Häst, lag'!$K$4</x:definedName>
+    <x:definedName name="klass" localSheetId="2">'Lag grund A'!$L$4</x:definedName>
+    <x:definedName name="klass" localSheetId="4">'Lag grund B'!$L$4</x:definedName>
+    <x:definedName name="klass" localSheetId="3">'Lag grund D'!$L$4</x:definedName>
+    <x:definedName name="klass" localSheetId="8">'Lag kür art'!$L$4</x:definedName>
+    <x:definedName name="klass" localSheetId="9">'Lag kür art senior'!$L$4</x:definedName>
+    <x:definedName name="klass" localSheetId="6">'Lag kür tekn junior'!$L$4</x:definedName>
+    <x:definedName name="klass" localSheetId="5">'Lag kür tekn mellan'!$L$4</x:definedName>
+    <x:definedName name="klass" localSheetId="7">'Lag kür tekn sr'!$L$4</x:definedName>
+    <x:definedName name="moment" localSheetId="1">'Häst, lag'!$K$5</x:definedName>
+    <x:definedName name="moment" localSheetId="2">'Lag grund A'!$L$5</x:definedName>
+    <x:definedName name="moment" localSheetId="4">'Lag grund B'!$L$5</x:definedName>
+    <x:definedName name="moment" localSheetId="3">'Lag grund D'!$L$5</x:definedName>
+    <x:definedName name="moment" localSheetId="8">'Lag kür art'!$L$5</x:definedName>
+    <x:definedName name="moment" localSheetId="9">'Lag kür art senior'!$L$5</x:definedName>
+    <x:definedName name="moment" localSheetId="6">'Lag kür tekn junior'!$L$5</x:definedName>
+    <x:definedName name="moment" localSheetId="5">'Lag kür tekn mellan'!$L$5</x:definedName>
+    <x:definedName name="moment" localSheetId="7">'Lag kür tekn sr'!$L$5</x:definedName>
+    <x:definedName name="result" localSheetId="1">'Häst, lag'!$K$32</x:definedName>
+    <x:definedName name="result" localSheetId="2">'Lag grund A'!$L$29</x:definedName>
+    <x:definedName name="result" localSheetId="4">'Lag grund B'!$L$29</x:definedName>
+    <x:definedName name="result" localSheetId="3">'Lag grund D'!$L$29</x:definedName>
+    <x:definedName name="result" localSheetId="8">'Lag kür art'!$L$24</x:definedName>
+    <x:definedName name="result" localSheetId="9">'Lag kür art senior'!$L$24</x:definedName>
+    <x:definedName name="result" localSheetId="6">'Lag kür tekn junior'!$L$34</x:definedName>
+    <x:definedName name="result" localSheetId="5">'Lag kür tekn mellan'!$L$34</x:definedName>
+    <x:definedName name="result" localSheetId="7">'Lag kür tekn sr'!$L$35</x:definedName>
+    <x:definedName name="_xlnm.Print_Area" localSheetId="1">'Häst, lag'!$A$1:$L$36</x:definedName>
+  </x:definedNames>
+  <x:calcPr calcId="191029"/>
+  <x:extLst>
+    <x:ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
       </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
-</workbook>
+    </x:ext>
+  </x:extLst>
+</x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4322,594 +4322,594 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84C25329-D17D-4FF2-BF65-A450782F317F}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:L36"/>
-  <sheetFormatPr defaultColWidth="9.06640625" defaultRowHeight="12.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="5.73046875" style="43" customWidth="1"/>
-    <col min="2" max="2" width="8.796875" style="43" customWidth="1"/>
-    <col min="3" max="3" width="10.265625" style="43" customWidth="1"/>
-    <col min="4" max="4" width="10.06640625" style="43" customWidth="1"/>
-    <col min="5" max="5" width="9.796875" style="43" customWidth="1"/>
-    <col min="6" max="7" width="9.9296875" style="43" customWidth="1"/>
-    <col min="8" max="8" width="6.265625" style="43" customWidth="1"/>
-    <col min="9" max="9" width="5.73046875" style="43" customWidth="1"/>
-    <col min="10" max="11" width="7.06640625" style="43" customWidth="1"/>
-    <col min="12" max="12" width="7.265625" style="43" customWidth="1"/>
-    <col min="13" max="16384" width="9.06640625" style="43"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:12" s="138" customFormat="1" ht="6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="1:12" s="138" customFormat="1" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="139" t="s">
-        <v>8</v>
-      </c>
-      <c r="G2" s="140"/>
-      <c r="H2" s="141" t="s">
-        <v>62</v>
-      </c>
-      <c r="I2" s="142"/>
-      <c r="J2" s="143"/>
-      <c r="K2" s="144"/>
-    </row>
-    <row r="3" spans="1:12" s="138" customFormat="1" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="145" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3" s="140"/>
-      <c r="H3" s="141" t="s">
-        <v>63</v>
-      </c>
-      <c r="I3" s="142"/>
-      <c r="J3" s="143"/>
-      <c r="K3" s="144"/>
-    </row>
-    <row r="4" spans="1:12" s="138" customFormat="1" ht="17.55" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="146" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="146"/>
-      <c r="C4" s="258"/>
-      <c r="D4" s="258"/>
-      <c r="E4" s="147"/>
-      <c r="G4" s="140"/>
-      <c r="H4" s="141" t="s">
-        <v>56</v>
-      </c>
-      <c r="I4" s="142"/>
-      <c r="J4" s="143"/>
-      <c r="K4" s="144"/>
-    </row>
-    <row r="5" spans="1:12" s="138" customFormat="1" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="148" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="148"/>
-      <c r="C5" s="256"/>
-      <c r="D5" s="256"/>
-      <c r="E5" s="256"/>
-      <c r="G5" s="140"/>
-      <c r="H5" s="141" t="s">
-        <v>10</v>
-      </c>
-      <c r="I5" s="149"/>
-      <c r="J5" s="143"/>
-      <c r="K5" s="144"/>
-    </row>
-    <row r="6" spans="1:12" s="138" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="148" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="148"/>
-      <c r="C6" s="256"/>
-      <c r="D6" s="256"/>
-      <c r="E6" s="256"/>
-      <c r="G6" s="138" t="s">
-        <v>15</v>
-      </c>
-      <c r="K6" s="150"/>
-    </row>
-    <row r="7" spans="1:12" s="138" customFormat="1" ht="17.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="148" t="s">
-        <v>61</v>
-      </c>
-      <c r="B7" s="148"/>
-      <c r="C7" s="151"/>
-      <c r="D7" s="151"/>
-      <c r="E7" s="151"/>
-      <c r="G7" s="146" t="s">
-        <v>0</v>
-      </c>
-      <c r="H7" s="259"/>
-      <c r="I7" s="260"/>
-      <c r="J7" s="260"/>
-      <c r="K7" s="260"/>
-    </row>
-    <row r="8" spans="1:12" s="138" customFormat="1" ht="17.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="146" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="146"/>
-      <c r="C8" s="259"/>
-      <c r="D8" s="259"/>
-      <c r="E8" s="259"/>
-      <c r="G8" s="148" t="s">
-        <v>1</v>
-      </c>
-      <c r="H8" s="256"/>
-      <c r="I8" s="257"/>
-      <c r="J8" s="257"/>
-      <c r="K8" s="257"/>
-    </row>
-    <row r="9" spans="1:12" s="138" customFormat="1" ht="17.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="148" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="148"/>
-      <c r="C9" s="256"/>
-      <c r="D9" s="256"/>
-      <c r="E9" s="256"/>
-      <c r="G9" s="148" t="s">
-        <v>2</v>
-      </c>
-      <c r="H9" s="256"/>
-      <c r="I9" s="257"/>
-      <c r="J9" s="257"/>
-      <c r="K9" s="257"/>
-    </row>
-    <row r="10" spans="1:12" s="138" customFormat="1" ht="17.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="148" t="s">
-        <v>59</v>
-      </c>
-      <c r="B10" s="148"/>
-      <c r="C10" s="256"/>
-      <c r="D10" s="256"/>
-      <c r="E10" s="256"/>
-      <c r="G10" s="148" t="s">
-        <v>3</v>
-      </c>
-      <c r="H10" s="256"/>
-      <c r="I10" s="257"/>
-      <c r="J10" s="257"/>
-      <c r="K10" s="257"/>
-    </row>
-    <row r="11" spans="1:12" s="138" customFormat="1" ht="17.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="G11" s="148" t="s">
-        <v>4</v>
-      </c>
-      <c r="H11" s="256"/>
-      <c r="I11" s="257"/>
-      <c r="J11" s="257"/>
-      <c r="K11" s="257"/>
-    </row>
-    <row r="12" spans="1:12" s="138" customFormat="1" ht="17.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C12" s="152"/>
-      <c r="G12" s="148" t="s">
-        <v>5</v>
-      </c>
-      <c r="H12" s="256"/>
-      <c r="I12" s="257"/>
-      <c r="J12" s="257"/>
-      <c r="K12" s="257"/>
-    </row>
-    <row r="13" spans="1:12" s="138" customFormat="1" ht="6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C13" s="152"/>
-      <c r="G13" s="153"/>
-      <c r="H13" s="154"/>
-      <c r="I13" s="153"/>
-      <c r="J13" s="153"/>
-      <c r="K13" s="153"/>
-    </row>
-    <row r="14" spans="1:12" ht="12.75" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="138"/>
-      <c r="B14" s="138"/>
-      <c r="C14" s="155"/>
-      <c r="D14" s="155"/>
-      <c r="E14" s="155"/>
-      <c r="F14" s="155"/>
-      <c r="G14" s="138"/>
-      <c r="H14" s="230" t="s">
-        <v>26</v>
-      </c>
-      <c r="I14" s="231"/>
-      <c r="J14" s="232" t="s">
-        <v>60</v>
-      </c>
-      <c r="K14" s="233"/>
-      <c r="L14" s="234"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A15" s="235" t="s">
-        <v>113</v>
-      </c>
-      <c r="B15" s="239" t="s">
-        <v>114</v>
-      </c>
-      <c r="C15" s="240"/>
-      <c r="D15" s="240"/>
-      <c r="E15" s="240"/>
-      <c r="F15" s="240"/>
-      <c r="G15" s="240"/>
-      <c r="H15" s="243"/>
-      <c r="I15" s="244"/>
-      <c r="J15" s="249" t="s">
-        <v>115</v>
-      </c>
-      <c r="K15" s="251">
-        <f>SUM(B20:G20)/6</f>
-        <v>0</v>
-      </c>
-      <c r="L15" s="253">
-        <f>ROUND(K15*0.6,3)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A16" s="236"/>
-      <c r="B16" s="241"/>
-      <c r="C16" s="242"/>
-      <c r="D16" s="242"/>
-      <c r="E16" s="242"/>
-      <c r="F16" s="242"/>
-      <c r="G16" s="242"/>
-      <c r="H16" s="245"/>
-      <c r="I16" s="246"/>
-      <c r="J16" s="217"/>
-      <c r="K16" s="252"/>
-      <c r="L16" s="254"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A17" s="236"/>
-      <c r="B17" s="241"/>
-      <c r="C17" s="242"/>
-      <c r="D17" s="242"/>
-      <c r="E17" s="242"/>
-      <c r="F17" s="242"/>
-      <c r="G17" s="242"/>
-      <c r="H17" s="245"/>
-      <c r="I17" s="246"/>
-      <c r="J17" s="217"/>
-      <c r="K17" s="252"/>
-      <c r="L17" s="254"/>
-    </row>
-    <row r="18" spans="1:12" ht="136.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="236"/>
-      <c r="B18" s="241"/>
-      <c r="C18" s="242"/>
-      <c r="D18" s="242"/>
-      <c r="E18" s="242"/>
-      <c r="F18" s="242"/>
-      <c r="G18" s="242"/>
-      <c r="H18" s="245"/>
-      <c r="I18" s="246"/>
-      <c r="J18" s="217"/>
-      <c r="K18" s="252"/>
-      <c r="L18" s="254"/>
-    </row>
-    <row r="19" spans="1:12" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="237"/>
-      <c r="B19" s="156" t="s">
-        <v>116</v>
-      </c>
-      <c r="C19" s="157" t="s">
-        <v>117</v>
-      </c>
-      <c r="D19" s="158" t="s">
-        <v>118</v>
-      </c>
-      <c r="E19" s="157" t="s">
-        <v>119</v>
-      </c>
-      <c r="F19" s="157" t="s">
-        <v>120</v>
-      </c>
-      <c r="G19" s="159" t="s">
-        <v>121</v>
-      </c>
-      <c r="H19" s="245"/>
-      <c r="I19" s="246"/>
-      <c r="J19" s="217"/>
-      <c r="K19" s="252"/>
-      <c r="L19" s="254"/>
-    </row>
-    <row r="20" spans="1:12" ht="28.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="238"/>
-      <c r="B20" s="160"/>
-      <c r="C20" s="161"/>
-      <c r="D20" s="161"/>
-      <c r="E20" s="161"/>
-      <c r="F20" s="161"/>
-      <c r="G20" s="162"/>
-      <c r="H20" s="247"/>
-      <c r="I20" s="248"/>
-      <c r="J20" s="250"/>
-      <c r="K20" s="252"/>
-      <c r="L20" s="255"/>
-    </row>
-    <row r="21" spans="1:12" ht="12.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="194"/>
-      <c r="B21" s="197" t="s">
-        <v>136</v>
-      </c>
-      <c r="C21" s="197"/>
-      <c r="D21" s="197"/>
-      <c r="E21" s="197"/>
-      <c r="F21" s="197"/>
-      <c r="G21" s="197"/>
-      <c r="H21" s="199"/>
-      <c r="I21" s="200"/>
-      <c r="J21" s="205" t="s">
-        <v>7</v>
-      </c>
-      <c r="K21" s="227">
-        <f>SUMPRODUCT(B26:G26,B25:G25)</f>
-        <v>0</v>
-      </c>
-      <c r="L21" s="208">
-        <f>IF((K21-K28)&gt;=0,ROUND((K21-K28)*0.25,3),0.000000000001)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A22" s="195"/>
-      <c r="B22" s="198"/>
-      <c r="C22" s="198"/>
-      <c r="D22" s="198"/>
-      <c r="E22" s="198"/>
-      <c r="F22" s="198"/>
-      <c r="G22" s="198"/>
-      <c r="H22" s="201"/>
-      <c r="I22" s="202"/>
-      <c r="J22" s="206"/>
-      <c r="K22" s="228"/>
-      <c r="L22" s="209"/>
-    </row>
-    <row r="23" spans="1:12" ht="53" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="195"/>
-      <c r="B23" s="198"/>
-      <c r="C23" s="198"/>
-      <c r="D23" s="198"/>
-      <c r="E23" s="198"/>
-      <c r="F23" s="198"/>
-      <c r="G23" s="198"/>
-      <c r="H23" s="201"/>
-      <c r="I23" s="202"/>
-      <c r="J23" s="206"/>
-      <c r="K23" s="228"/>
-      <c r="L23" s="209"/>
-    </row>
-    <row r="24" spans="1:12" ht="15.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="195"/>
-      <c r="B24" s="219" t="s">
-        <v>133</v>
-      </c>
-      <c r="C24" s="220"/>
-      <c r="D24" s="221" t="s">
-        <v>134</v>
-      </c>
-      <c r="E24" s="222"/>
-      <c r="F24" s="223" t="s">
-        <v>135</v>
-      </c>
-      <c r="G24" s="224"/>
-      <c r="H24" s="201"/>
-      <c r="I24" s="202"/>
-      <c r="J24" s="206"/>
-      <c r="K24" s="228"/>
-      <c r="L24" s="209"/>
-    </row>
-    <row r="25" spans="1:12" ht="13.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="195"/>
-      <c r="B25" s="225">
-        <v>0.5</v>
-      </c>
-      <c r="C25" s="226"/>
-      <c r="D25" s="181">
-        <v>0.25</v>
-      </c>
-      <c r="E25" s="182"/>
-      <c r="F25" s="183">
-        <v>0.25</v>
-      </c>
-      <c r="G25" s="184"/>
-      <c r="H25" s="201"/>
-      <c r="I25" s="202"/>
-      <c r="J25" s="206"/>
-      <c r="K25" s="228"/>
-      <c r="L25" s="209"/>
-    </row>
-    <row r="26" spans="1:12" ht="28.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="195"/>
-      <c r="B26" s="185"/>
-      <c r="C26" s="186"/>
-      <c r="D26" s="187"/>
-      <c r="E26" s="188"/>
-      <c r="F26" s="186"/>
-      <c r="G26" s="189"/>
-      <c r="H26" s="201"/>
-      <c r="I26" s="202"/>
-      <c r="J26" s="206"/>
-      <c r="K26" s="229"/>
-      <c r="L26" s="209"/>
-    </row>
-    <row r="27" spans="1:12" ht="10.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="195"/>
-      <c r="B27" s="177"/>
-      <c r="C27" s="178"/>
-      <c r="D27" s="179"/>
-      <c r="E27" s="179"/>
-      <c r="F27" s="178"/>
-      <c r="G27" s="180"/>
-      <c r="H27" s="201"/>
-      <c r="I27" s="202"/>
-      <c r="J27" s="206"/>
-      <c r="K27" s="176"/>
-      <c r="L27" s="209"/>
-    </row>
-    <row r="28" spans="1:12" ht="28.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="196"/>
-      <c r="B28" s="163" t="s">
-        <v>122</v>
-      </c>
-      <c r="C28" s="164"/>
-      <c r="D28" s="164"/>
-      <c r="E28" s="164"/>
-      <c r="F28" s="164"/>
-      <c r="G28" s="164"/>
-      <c r="H28" s="203"/>
-      <c r="I28" s="204"/>
-      <c r="J28" s="207"/>
-      <c r="K28" s="165">
-        <f>SUM(C28:G28)</f>
-        <v>0</v>
-      </c>
-      <c r="L28" s="210"/>
-    </row>
-    <row r="29" spans="1:12" ht="114.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="194" t="s">
-        <v>16</v>
-      </c>
-      <c r="B29" s="197" t="s">
-        <v>137</v>
-      </c>
-      <c r="C29" s="211"/>
-      <c r="D29" s="211"/>
-      <c r="E29" s="211"/>
-      <c r="F29" s="211"/>
-      <c r="G29" s="212"/>
-      <c r="H29" s="213"/>
-      <c r="I29" s="214"/>
-      <c r="J29" s="217" t="s">
-        <v>123</v>
-      </c>
-      <c r="K29" s="166">
-        <v>0</v>
-      </c>
-      <c r="L29" s="190">
-        <f>IF((K29-K30)&gt;=0,ROUND((K29-K30)*0.15,3),0.00000000001)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" ht="28.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="196"/>
-      <c r="B30" s="167" t="s">
-        <v>122</v>
-      </c>
-      <c r="C30" s="164"/>
-      <c r="D30" s="164"/>
-      <c r="E30" s="164"/>
-      <c r="F30" s="164"/>
-      <c r="G30" s="164"/>
-      <c r="H30" s="215"/>
-      <c r="I30" s="216"/>
-      <c r="J30" s="218"/>
-      <c r="K30" s="165">
-        <f>SUM(C30:G30)</f>
-        <v>0</v>
-      </c>
-      <c r="L30" s="191"/>
-    </row>
-    <row r="31" spans="1:12" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A31" s="44"/>
-      <c r="B31" s="44"/>
-      <c r="C31" s="44"/>
-      <c r="D31" s="44"/>
-      <c r="E31" s="44"/>
-      <c r="F31" s="44"/>
-      <c r="G31" s="44"/>
-      <c r="H31" s="44"/>
-      <c r="K31" s="57"/>
-    </row>
-    <row r="32" spans="1:12" ht="28.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="I32" s="45" t="s">
-        <v>9</v>
-      </c>
-      <c r="J32" s="46"/>
-      <c r="K32" s="192">
-        <f>SUM(L15:L29)</f>
-        <v>0</v>
-      </c>
-      <c r="L32" s="193"/>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A36" s="169" t="s">
-        <v>18</v>
-      </c>
-      <c r="B36" s="169"/>
-      <c r="C36" s="169"/>
-      <c r="D36" s="169"/>
-      <c r="E36" s="169"/>
-      <c r="F36" s="168"/>
-      <c r="G36" s="138"/>
-      <c r="H36" s="146" t="s">
-        <v>19</v>
-      </c>
-      <c r="I36" s="146"/>
-      <c r="J36" s="146"/>
-      <c r="K36" s="146"/>
-      <c r="L36" s="146"/>
-    </row>
-  </sheetData>
-  <mergeCells count="41">
-    <mergeCell ref="H12:K12"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="C6:E6"/>
-    <mergeCell ref="H7:K7"/>
-    <mergeCell ref="C8:E8"/>
-    <mergeCell ref="H8:K8"/>
-    <mergeCell ref="C9:E9"/>
-    <mergeCell ref="H9:K9"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="H10:K10"/>
-    <mergeCell ref="H11:K11"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="J14:L14"/>
-    <mergeCell ref="A15:A20"/>
-    <mergeCell ref="B15:G18"/>
-    <mergeCell ref="H15:I20"/>
-    <mergeCell ref="J15:J20"/>
-    <mergeCell ref="K15:K20"/>
-    <mergeCell ref="L15:L20"/>
-    <mergeCell ref="L29:L30"/>
-    <mergeCell ref="K32:L32"/>
-    <mergeCell ref="A21:A28"/>
-    <mergeCell ref="B21:G23"/>
-    <mergeCell ref="H21:I28"/>
-    <mergeCell ref="J21:J28"/>
-    <mergeCell ref="L21:L28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="B29:G29"/>
-    <mergeCell ref="H29:I30"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="K21:K26"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="F26:G26"/>
-  </mergeCells>
-  <dataValidations count="1">
-    <dataValidation type="decimal" operator="lessThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Endast siffror giltiga" error="Ej giltig siffra_x000a_Kan du ha skrivit komma  istället för punkt eller tvärt om" sqref="C30:G30 C28 D28 E28 F28 G28 F26:G26 D26:E26 B26:C26 K29 B20 C20 D20 E20 F20 G20" xr:uid="{717696C7-3684-477B-A49A-9E6458A0FA01}">
-      <formula1>11</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.47244094488188981" right="0.15748031496062992" top="0.98425196850393704" bottom="0.39370078740157483" header="0.43307086614173229" footer="0.19685039370078741"/>
-  <pageSetup paperSize="9" scale="90" orientation="portrait" r:id="rId1"/>
-  <headerFooter alignWithMargins="0">
-    <oddHeader>&amp;L&amp;G
-&amp;C&amp;"Verdana,Normal"&amp;12PROTOKOLL FÖR LAGTÄVLAN</oddHeader>
-    <oddFooter>&amp;R2025-03-16</oddFooter>
-  </headerFooter>
-  <legacyDrawingHF r:id="rId2"/>
-</worksheet>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xr:uid="{84C25329-D17D-4FF2-BF65-A450782F317F}" mc:Ignorable="x14ac xr xr2 xr3">
+  <x:sheetPr>
+    <x:pageSetUpPr fitToPage="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:L36"/>
+  <x:sheetFormatPr defaultColWidth="9.06640625" defaultRowHeight="12.4" x14ac:dyDescent="0.3"/>
+  <x:cols>
+    <x:col min="1" max="1" width="5.73046875" style="43" customWidth="1"/>
+    <x:col min="2" max="2" width="8.796875" style="43" customWidth="1"/>
+    <x:col min="3" max="3" width="10.265625" style="43" customWidth="1"/>
+    <x:col min="4" max="4" width="10.06640625" style="43" customWidth="1"/>
+    <x:col min="5" max="5" width="9.796875" style="43" customWidth="1"/>
+    <x:col min="6" max="7" width="9.9296875" style="43" customWidth="1"/>
+    <x:col min="8" max="8" width="6.265625" style="43" customWidth="1"/>
+    <x:col min="9" max="9" width="5.73046875" style="43" customWidth="1"/>
+    <x:col min="10" max="11" width="7.06640625" style="43" customWidth="1"/>
+    <x:col min="12" max="12" width="7.265625" style="43" customWidth="1"/>
+    <x:col min="13" max="16384" width="9.06640625" style="43"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:12" s="138" customFormat="1" ht="6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <x:row r="2" spans="1:12" s="138" customFormat="1" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <x:c r="A2" s="139" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G2" s="140"/>
+      <x:c r="H2" s="141" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="I2" s="142"/>
+      <x:c r="J2" s="143"/>
+      <x:c r="K2" s="144"/>
+    </x:row>
+    <x:row r="3" spans="1:12" s="138" customFormat="1" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <x:c r="A3" s="145" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="G3" s="140"/>
+      <x:c r="H3" s="141" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="I3" s="142"/>
+      <x:c r="J3" s="143"/>
+      <x:c r="K3" s="144"/>
+    </x:row>
+    <x:row r="4" spans="1:12" s="138" customFormat="1" ht="17.55" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <x:c r="A4" s="146" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B4" s="146"/>
+      <x:c r="C4" s="258"/>
+      <x:c r="D4" s="258"/>
+      <x:c r="E4" s="147"/>
+      <x:c r="G4" s="140"/>
+      <x:c r="H4" s="141" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="I4" s="142"/>
+      <x:c r="J4" s="143"/>
+      <x:c r="K4" s="144"/>
+    </x:row>
+    <x:row r="5" spans="1:12" s="138" customFormat="1" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <x:c r="A5" s="148" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B5" s="148"/>
+      <x:c r="C5" s="256"/>
+      <x:c r="D5" s="256"/>
+      <x:c r="E5" s="256"/>
+      <x:c r="G5" s="140"/>
+      <x:c r="H5" s="141" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="I5" s="149"/>
+      <x:c r="J5" s="143"/>
+      <x:c r="K5" s="144"/>
+    </x:row>
+    <x:row r="6" spans="1:12" s="138" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.3">
+      <x:c r="A6" s="148" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B6" s="148"/>
+      <x:c r="C6" s="256"/>
+      <x:c r="D6" s="256"/>
+      <x:c r="E6" s="256"/>
+      <x:c r="G6" s="138" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="K6" s="150"/>
+    </x:row>
+    <x:row r="7" spans="1:12" s="138" customFormat="1" ht="17.2" customHeight="1" x14ac:dyDescent="0.3">
+      <x:c r="A7" s="148" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="B7" s="148"/>
+      <x:c r="C7" s="151"/>
+      <x:c r="D7" s="151"/>
+      <x:c r="E7" s="151"/>
+      <x:c r="G7" s="146" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H7" s="259"/>
+      <x:c r="I7" s="260"/>
+      <x:c r="J7" s="260"/>
+      <x:c r="K7" s="260"/>
+    </x:row>
+    <x:row r="8" spans="1:12" s="138" customFormat="1" ht="17.2" customHeight="1" x14ac:dyDescent="0.3">
+      <x:c r="A8" s="146" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B8" s="146"/>
+      <x:c r="C8" s="259"/>
+      <x:c r="D8" s="259"/>
+      <x:c r="E8" s="259"/>
+      <x:c r="G8" s="148" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H8" s="256"/>
+      <x:c r="I8" s="257"/>
+      <x:c r="J8" s="257"/>
+      <x:c r="K8" s="257"/>
+    </x:row>
+    <x:row r="9" spans="1:12" s="138" customFormat="1" ht="17.2" customHeight="1" x14ac:dyDescent="0.3">
+      <x:c r="A9" s="148" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B9" s="148"/>
+      <x:c r="C9" s="256"/>
+      <x:c r="D9" s="256"/>
+      <x:c r="E9" s="256"/>
+      <x:c r="G9" s="148" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H9" s="256"/>
+      <x:c r="I9" s="257"/>
+      <x:c r="J9" s="257"/>
+      <x:c r="K9" s="257"/>
+    </x:row>
+    <x:row r="10" spans="1:12" s="138" customFormat="1" ht="17.2" customHeight="1" x14ac:dyDescent="0.3">
+      <x:c r="A10" s="148" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B10" s="148"/>
+      <x:c r="C10" s="256"/>
+      <x:c r="D10" s="256"/>
+      <x:c r="E10" s="256"/>
+      <x:c r="G10" s="148" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H10" s="256"/>
+      <x:c r="I10" s="257"/>
+      <x:c r="J10" s="257"/>
+      <x:c r="K10" s="257"/>
+    </x:row>
+    <x:row r="11" spans="1:12" s="138" customFormat="1" ht="17.2" customHeight="1" x14ac:dyDescent="0.3">
+      <x:c r="G11" s="148" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H11" s="256"/>
+      <x:c r="I11" s="257"/>
+      <x:c r="J11" s="257"/>
+      <x:c r="K11" s="257"/>
+    </x:row>
+    <x:row r="12" spans="1:12" s="138" customFormat="1" ht="17.2" customHeight="1" x14ac:dyDescent="0.3">
+      <x:c r="C12" s="152"/>
+      <x:c r="G12" s="148" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H12" s="256"/>
+      <x:c r="I12" s="257"/>
+      <x:c r="J12" s="257"/>
+      <x:c r="K12" s="257"/>
+    </x:row>
+    <x:row r="13" spans="1:12" s="138" customFormat="1" ht="6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <x:c r="C13" s="152"/>
+      <x:c r="G13" s="153"/>
+      <x:c r="H13" s="154"/>
+      <x:c r="I13" s="153"/>
+      <x:c r="J13" s="153"/>
+      <x:c r="K13" s="153"/>
+    </x:row>
+    <x:row r="14" spans="1:12" ht="12.75" thickBot="1" x14ac:dyDescent="0.35">
+      <x:c r="A14" s="138"/>
+      <x:c r="B14" s="138"/>
+      <x:c r="C14" s="155"/>
+      <x:c r="D14" s="155"/>
+      <x:c r="E14" s="155"/>
+      <x:c r="F14" s="155"/>
+      <x:c r="G14" s="138"/>
+      <x:c r="H14" s="230" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="I14" s="231"/>
+      <x:c r="J14" s="232" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="K14" s="233"/>
+      <x:c r="L14" s="234"/>
+    </x:row>
+    <x:row r="15" spans="1:12" x14ac:dyDescent="0.3">
+      <x:c r="A15" s="235" t="s">
+        <x:v>113</x:v>
+      </x:c>
+      <x:c r="B15" s="239" t="s">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="C15" s="240"/>
+      <x:c r="D15" s="240"/>
+      <x:c r="E15" s="240"/>
+      <x:c r="F15" s="240"/>
+      <x:c r="G15" s="240"/>
+      <x:c r="H15" s="243"/>
+      <x:c r="I15" s="244"/>
+      <x:c r="J15" s="249" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="K15" s="251">
+        <x:f>SUM(B20:G20)/6</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L15" s="253">
+        <x:f>ROUND(K15*0.6,3)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" spans="1:12" x14ac:dyDescent="0.3">
+      <x:c r="A16" s="236"/>
+      <x:c r="B16" s="241"/>
+      <x:c r="C16" s="242"/>
+      <x:c r="D16" s="242"/>
+      <x:c r="E16" s="242"/>
+      <x:c r="F16" s="242"/>
+      <x:c r="G16" s="242"/>
+      <x:c r="H16" s="245"/>
+      <x:c r="I16" s="246"/>
+      <x:c r="J16" s="217"/>
+      <x:c r="K16" s="252"/>
+      <x:c r="L16" s="254"/>
+    </x:row>
+    <x:row r="17" spans="1:12" x14ac:dyDescent="0.3">
+      <x:c r="A17" s="236"/>
+      <x:c r="B17" s="241"/>
+      <x:c r="C17" s="242"/>
+      <x:c r="D17" s="242"/>
+      <x:c r="E17" s="242"/>
+      <x:c r="F17" s="242"/>
+      <x:c r="G17" s="242"/>
+      <x:c r="H17" s="245"/>
+      <x:c r="I17" s="246"/>
+      <x:c r="J17" s="217"/>
+      <x:c r="K17" s="252"/>
+      <x:c r="L17" s="254"/>
+    </x:row>
+    <x:row r="18" spans="1:12" ht="136.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <x:c r="A18" s="236"/>
+      <x:c r="B18" s="241"/>
+      <x:c r="C18" s="242"/>
+      <x:c r="D18" s="242"/>
+      <x:c r="E18" s="242"/>
+      <x:c r="F18" s="242"/>
+      <x:c r="G18" s="242"/>
+      <x:c r="H18" s="245"/>
+      <x:c r="I18" s="246"/>
+      <x:c r="J18" s="217"/>
+      <x:c r="K18" s="252"/>
+      <x:c r="L18" s="254"/>
+    </x:row>
+    <x:row r="19" spans="1:12" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <x:c r="A19" s="237"/>
+      <x:c r="B19" s="156" t="s">
+        <x:v>116</x:v>
+      </x:c>
+      <x:c r="C19" s="157" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="D19" s="158" t="s">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="E19" s="157" t="s">
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="F19" s="157" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="G19" s="159" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="H19" s="245"/>
+      <x:c r="I19" s="246"/>
+      <x:c r="J19" s="217"/>
+      <x:c r="K19" s="252"/>
+      <x:c r="L19" s="254"/>
+    </x:row>
+    <x:row r="20" spans="1:12" ht="28.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <x:c r="A20" s="238"/>
+      <x:c r="B20" s="160"/>
+      <x:c r="C20" s="161"/>
+      <x:c r="D20" s="161"/>
+      <x:c r="E20" s="161"/>
+      <x:c r="F20" s="161"/>
+      <x:c r="G20" s="162"/>
+      <x:c r="H20" s="247"/>
+      <x:c r="I20" s="248"/>
+      <x:c r="J20" s="250"/>
+      <x:c r="K20" s="252"/>
+      <x:c r="L20" s="255"/>
+    </x:row>
+    <x:row r="21" spans="1:12" ht="12.4" customHeight="1" x14ac:dyDescent="0.3">
+      <x:c r="A21" s="194"/>
+      <x:c r="B21" s="197" t="s">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="C21" s="197"/>
+      <x:c r="D21" s="197"/>
+      <x:c r="E21" s="197"/>
+      <x:c r="F21" s="197"/>
+      <x:c r="G21" s="197"/>
+      <x:c r="H21" s="199"/>
+      <x:c r="I21" s="200"/>
+      <x:c r="J21" s="205" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="K21" s="227">
+        <x:f>SUMPRODUCT(B26:G26,B25:G25)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L21" s="208">
+        <x:f>IF((K21-K28)&gt;=0,ROUND((K21-K28)*0.25,3),0.000000000001)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" spans="1:12" x14ac:dyDescent="0.3">
+      <x:c r="A22" s="195"/>
+      <x:c r="B22" s="198"/>
+      <x:c r="C22" s="198"/>
+      <x:c r="D22" s="198"/>
+      <x:c r="E22" s="198"/>
+      <x:c r="F22" s="198"/>
+      <x:c r="G22" s="198"/>
+      <x:c r="H22" s="201"/>
+      <x:c r="I22" s="202"/>
+      <x:c r="J22" s="206"/>
+      <x:c r="K22" s="228"/>
+      <x:c r="L22" s="209"/>
+    </x:row>
+    <x:row r="23" spans="1:12" ht="53" customHeight="1" x14ac:dyDescent="0.3">
+      <x:c r="A23" s="195"/>
+      <x:c r="B23" s="198"/>
+      <x:c r="C23" s="198"/>
+      <x:c r="D23" s="198"/>
+      <x:c r="E23" s="198"/>
+      <x:c r="F23" s="198"/>
+      <x:c r="G23" s="198"/>
+      <x:c r="H23" s="201"/>
+      <x:c r="I23" s="202"/>
+      <x:c r="J23" s="206"/>
+      <x:c r="K23" s="228"/>
+      <x:c r="L23" s="209"/>
+    </x:row>
+    <x:row r="24" spans="1:12" ht="15.4" customHeight="1" x14ac:dyDescent="0.3">
+      <x:c r="A24" s="195"/>
+      <x:c r="B24" s="219" t="s">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="C24" s="220"/>
+      <x:c r="D24" s="221" t="s">
+        <x:v>134</x:v>
+      </x:c>
+      <x:c r="E24" s="222"/>
+      <x:c r="F24" s="223" t="s">
+        <x:v>135</x:v>
+      </x:c>
+      <x:c r="G24" s="224"/>
+      <x:c r="H24" s="201"/>
+      <x:c r="I24" s="202"/>
+      <x:c r="J24" s="206"/>
+      <x:c r="K24" s="228"/>
+      <x:c r="L24" s="209"/>
+    </x:row>
+    <x:row r="25" spans="1:12" ht="13.9" customHeight="1" x14ac:dyDescent="0.3">
+      <x:c r="A25" s="195"/>
+      <x:c r="B25" s="225">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C25" s="226"/>
+      <x:c r="D25" s="181">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="E25" s="182"/>
+      <x:c r="F25" s="183">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="G25" s="184"/>
+      <x:c r="H25" s="201"/>
+      <x:c r="I25" s="202"/>
+      <x:c r="J25" s="206"/>
+      <x:c r="K25" s="228"/>
+      <x:c r="L25" s="209"/>
+    </x:row>
+    <x:row r="26" spans="1:12" ht="28.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <x:c r="A26" s="195"/>
+      <x:c r="B26" s="185"/>
+      <x:c r="C26" s="186"/>
+      <x:c r="D26" s="187"/>
+      <x:c r="E26" s="188"/>
+      <x:c r="F26" s="186"/>
+      <x:c r="G26" s="189"/>
+      <x:c r="H26" s="201"/>
+      <x:c r="I26" s="202"/>
+      <x:c r="J26" s="206"/>
+      <x:c r="K26" s="229"/>
+      <x:c r="L26" s="209"/>
+    </x:row>
+    <x:row r="27" spans="1:12" ht="10.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <x:c r="A27" s="195"/>
+      <x:c r="B27" s="177"/>
+      <x:c r="C27" s="178"/>
+      <x:c r="D27" s="179"/>
+      <x:c r="E27" s="179"/>
+      <x:c r="F27" s="178"/>
+      <x:c r="G27" s="180"/>
+      <x:c r="H27" s="201"/>
+      <x:c r="I27" s="202"/>
+      <x:c r="J27" s="206"/>
+      <x:c r="K27" s="176"/>
+      <x:c r="L27" s="209"/>
+    </x:row>
+    <x:row r="28" spans="1:12" ht="28.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <x:c r="A28" s="196"/>
+      <x:c r="B28" s="163" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="C28" s="164"/>
+      <x:c r="D28" s="164"/>
+      <x:c r="E28" s="164"/>
+      <x:c r="F28" s="164"/>
+      <x:c r="G28" s="164"/>
+      <x:c r="H28" s="203"/>
+      <x:c r="I28" s="204"/>
+      <x:c r="J28" s="207"/>
+      <x:c r="K28" s="165">
+        <x:f>SUM(C28:G28)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L28" s="210"/>
+    </x:row>
+    <x:row r="29" spans="1:12" ht="114.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <x:c r="A29" s="194" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B29" s="197" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="C29" s="211"/>
+      <x:c r="D29" s="211"/>
+      <x:c r="E29" s="211"/>
+      <x:c r="F29" s="211"/>
+      <x:c r="G29" s="212"/>
+      <x:c r="H29" s="213"/>
+      <x:c r="I29" s="214"/>
+      <x:c r="J29" s="217" t="s">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="K29" s="166">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L29" s="190">
+        <x:f>IF((K29-K30)&gt;=0,ROUND((K29-K30)*0.15,3),0.00000000001)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" spans="1:12" ht="28.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <x:c r="A30" s="196"/>
+      <x:c r="B30" s="167" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="C30" s="164"/>
+      <x:c r="D30" s="164"/>
+      <x:c r="E30" s="164"/>
+      <x:c r="F30" s="164"/>
+      <x:c r="G30" s="164"/>
+      <x:c r="H30" s="215"/>
+      <x:c r="I30" s="216"/>
+      <x:c r="J30" s="218"/>
+      <x:c r="K30" s="165">
+        <x:f>SUM(C30:G30)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L30" s="191"/>
+    </x:row>
+    <x:row r="31" spans="1:12" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
+      <x:c r="A31" s="44"/>
+      <x:c r="B31" s="44"/>
+      <x:c r="C31" s="44"/>
+      <x:c r="D31" s="44"/>
+      <x:c r="E31" s="44"/>
+      <x:c r="F31" s="44"/>
+      <x:c r="G31" s="44"/>
+      <x:c r="H31" s="44"/>
+      <x:c r="K31" s="57"/>
+    </x:row>
+    <x:row r="32" spans="1:12" ht="28.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <x:c r="I32" s="45" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="J32" s="46"/>
+      <x:c r="K32" s="192">
+        <x:f>SUM(L15:L29)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L32" s="193"/>
+    </x:row>
+    <x:row r="36" spans="1:12" x14ac:dyDescent="0.3">
+      <x:c r="A36" s="169" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B36" s="169"/>
+      <x:c r="C36" s="169"/>
+      <x:c r="D36" s="169"/>
+      <x:c r="E36" s="169"/>
+      <x:c r="F36" s="168"/>
+      <x:c r="G36" s="138"/>
+      <x:c r="H36" s="146" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="I36" s="146"/>
+      <x:c r="J36" s="146"/>
+      <x:c r="K36" s="146"/>
+      <x:c r="L36" s="146"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells count="41">
+    <x:mergeCell ref="H12:K12"/>
+    <x:mergeCell ref="C4:D4"/>
+    <x:mergeCell ref="C5:E5"/>
+    <x:mergeCell ref="C6:E6"/>
+    <x:mergeCell ref="H7:K7"/>
+    <x:mergeCell ref="C8:E8"/>
+    <x:mergeCell ref="H8:K8"/>
+    <x:mergeCell ref="C9:E9"/>
+    <x:mergeCell ref="H9:K9"/>
+    <x:mergeCell ref="C10:E10"/>
+    <x:mergeCell ref="H10:K10"/>
+    <x:mergeCell ref="H11:K11"/>
+    <x:mergeCell ref="H14:I14"/>
+    <x:mergeCell ref="J14:L14"/>
+    <x:mergeCell ref="A15:A20"/>
+    <x:mergeCell ref="B15:G18"/>
+    <x:mergeCell ref="H15:I20"/>
+    <x:mergeCell ref="J15:J20"/>
+    <x:mergeCell ref="K15:K20"/>
+    <x:mergeCell ref="L15:L20"/>
+    <x:mergeCell ref="L29:L30"/>
+    <x:mergeCell ref="K32:L32"/>
+    <x:mergeCell ref="A21:A28"/>
+    <x:mergeCell ref="B21:G23"/>
+    <x:mergeCell ref="H21:I28"/>
+    <x:mergeCell ref="J21:J28"/>
+    <x:mergeCell ref="L21:L28"/>
+    <x:mergeCell ref="A29:A30"/>
+    <x:mergeCell ref="B29:G29"/>
+    <x:mergeCell ref="H29:I30"/>
+    <x:mergeCell ref="J29:J30"/>
+    <x:mergeCell ref="B24:C24"/>
+    <x:mergeCell ref="D24:E24"/>
+    <x:mergeCell ref="F24:G24"/>
+    <x:mergeCell ref="B25:C25"/>
+    <x:mergeCell ref="K21:K26"/>
+    <x:mergeCell ref="D25:E25"/>
+    <x:mergeCell ref="F25:G25"/>
+    <x:mergeCell ref="B26:C26"/>
+    <x:mergeCell ref="D26:E26"/>
+    <x:mergeCell ref="F26:G26"/>
+  </x:mergeCells>
+  <x:dataValidations count="1">
+    <x:dataValidation type="decimal" operator="lessThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Endast siffror giltiga" error="Ej giltig siffra_x000a_Kan du ha skrivit komma  istället för punkt eller tvärt om" sqref="C30:G30 C28 D28 E28 F28 G28 F26:G26 D26:E26 B26:C26 K29 B20 C20 D20 E20 F20 G20" xr:uid="{717696C7-3684-477B-A49A-9E6458A0FA01}">
+      <x:formula1>11</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.47244094488188981" right="0.15748031496062992" top="0.98425196850393704" bottom="0.39370078740157483" header="0.43307086614173229" footer="0.19685039370078741"/>
+  <x:pageSetup paperSize="9" scale="90" orientation="portrait" r:id="rId1"/>
+  <x:headerFooter alignWithMargins="0">
+    <x:oddHeader>&amp;L&amp;G
+&amp;C&amp;"Verdana,Normal"&amp;12PROTOKOLL FÖR LAGTÄVLAN</x:oddHeader>
+    <x:oddFooter>&amp;R2025-03-16</x:oddFooter>
+  </x:headerFooter>
+  <x:legacyDrawingHF r:id="rId2"/>
+</x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>